<commit_message>
ocr/nlp validation et rejet
</commit_message>
<xml_diff>
--- a/fiche_de_stage/Estimation Fiche de stage - ETU003346.xlsx
+++ b/fiche_de_stage/Estimation Fiche de stage - ETU003346.xlsx
@@ -14,10 +14,7 @@
     <sheet name="Estimation Agile info 4" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Estimation binome" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Estimation recrutement'!$A$3:$C$93</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Estimation recrutement'!$A$1:$C$93</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
@@ -28,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="35">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -207,8 +204,43 @@
       <color rgb="00274E13"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="39">
     <fill>
       <patternFill/>
     </fill>
@@ -401,8 +433,38 @@
         <fgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+        <bgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF3F8"/>
+        <bgColor rgb="00EAF3F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F6FA"/>
+        <bgColor rgb="00F2F6FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+        <bgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="27">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -693,11 +755,45 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="medium">
+        <color rgb="001F4E78"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0C4DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0C4DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0C4DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0C4DE"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0C4DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0C4DE"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="double">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17"/>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1079,6 +1175,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="34" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="34" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="35" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="32" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="36" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="31" fillId="36" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="37" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="38" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="34" fillId="38" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2847,1044 +2970,1078 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" style="77" min="1" max="1"/>
-    <col width="72" customWidth="1" style="77" min="2" max="2"/>
-    <col width="14" customWidth="1" style="77" min="3" max="3"/>
+    <col width="78" customWidth="1" style="77" min="2" max="2"/>
+    <col width="15" customWidth="1" style="77" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" s="77">
-      <c r="A1" s="148" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
         <is>
           <t>ESTIMATION DE STAGE ETU003346</t>
         </is>
       </c>
-      <c r="B1" s="166" t="n"/>
-      <c r="C1" s="166" t="n"/>
-    </row>
-    <row r="2" ht="24" customHeight="1" s="77">
-      <c r="A2" s="150" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
         <is>
           <t>Estimation en jours</t>
         </is>
       </c>
-      <c r="B2" s="167" t="n"/>
-      <c r="C2" s="168" t="n"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" s="77">
-      <c r="A3" s="152" t="n"/>
-      <c r="B3" s="152" t="inlineStr">
+    </row>
+    <row r="3">
+      <c r="A3" s="171" t="n"/>
+      <c r="B3" s="172" t="inlineStr">
         <is>
           <t>Tâches</t>
         </is>
       </c>
-      <c r="C3" s="152" t="inlineStr">
+      <c r="C3" s="173" t="inlineStr">
         <is>
           <t>Estimation</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1" s="77">
-      <c r="A4" s="153" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="174" t="inlineStr">
         <is>
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="B4" s="154" t="inlineStr">
+      <c r="B4" s="174" t="inlineStr">
         <is>
           <t>Analyse, cadrage et conception</t>
         </is>
       </c>
-      <c r="C4" s="153" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1" s="77">
-      <c r="A5" s="151" t="n"/>
-      <c r="B5" s="151" t="inlineStr">
+      <c r="C4" s="174" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="175" t="n"/>
+      <c r="B5" s="175" t="inlineStr">
         <is>
           <t>Analyse du cahier des charges et définition du périmètre V1</t>
         </is>
       </c>
-      <c r="C5" s="155" t="n">
+      <c r="C5" s="176" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1" s="77">
-      <c r="A6" s="151" t="n"/>
-      <c r="B6" s="151" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="175" t="n"/>
+      <c r="B6" s="175" t="inlineStr">
         <is>
           <t>Identification des modules fonctionnels du recrutement</t>
         </is>
       </c>
-      <c r="C6" s="155" t="n">
+      <c r="C6" s="176" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1" s="77">
-      <c r="A7" s="151" t="n"/>
-      <c r="B7" s="151" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="175" t="n"/>
+      <c r="B7" s="175" t="inlineStr">
         <is>
           <t>Analyse des parcours candidat / RH / admin</t>
         </is>
       </c>
-      <c r="C7" s="155" t="n">
+      <c r="C7" s="176" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1" s="77">
-      <c r="A8" s="151" t="n"/>
-      <c r="B8" s="151" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="175" t="n"/>
+      <c r="B8" s="175" t="inlineStr">
         <is>
           <t>Conception du MCD / MLD et des règles métier</t>
         </is>
       </c>
-      <c r="C8" s="155" t="n">
+      <c r="C8" s="176" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1" s="77">
-      <c r="A9" s="151" t="n"/>
-      <c r="B9" s="151" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="175" t="n"/>
+      <c r="B9" s="175" t="inlineStr">
         <is>
           <t>Conception de l'architecture Laravel / React / PostgreSQL / FastAPI</t>
         </is>
       </c>
-      <c r="C9" s="155" t="n">
+      <c r="C9" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="175" t="n"/>
+      <c r="B10" s="175" t="inlineStr">
+        <is>
+          <t>Planification du projet et préparation de l'environnement</t>
+        </is>
+      </c>
+      <c r="C10" s="176" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1" s="77">
-      <c r="A10" s="151" t="n"/>
-      <c r="B10" s="151" t="inlineStr">
-        <is>
-          <t>Planification du projet et préparation de l'environnement</t>
-        </is>
-      </c>
-      <c r="C10" s="155" t="n">
+    <row r="11">
+      <c r="A11" s="177" t="n"/>
+      <c r="B11" s="177" t="inlineStr">
+        <is>
+          <t>Sous-total</t>
+        </is>
+      </c>
+      <c r="C11" s="178">
+        <f>SUM(C5:C10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="174" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="B12" s="174" t="inlineStr">
+        <is>
+          <t>Socle technique, sécurité et référentiels de base</t>
+        </is>
+      </c>
+      <c r="C12" s="174" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="179" t="n"/>
+      <c r="B13" s="179" t="inlineStr">
+        <is>
+          <t>BACK-OFFICE / API</t>
+        </is>
+      </c>
+      <c r="C13" s="179" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="175" t="n"/>
+      <c r="B14" s="175" t="inlineStr">
+        <is>
+          <t>Configuration du projet Laravel et de l'environnement PostgreSQL</t>
+        </is>
+      </c>
+      <c r="C14" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="175" t="n"/>
+      <c r="B15" s="175" t="inlineStr">
+        <is>
+          <t>Mise en place des migrations principales et des seeders</t>
+        </is>
+      </c>
+      <c r="C15" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="175" t="n"/>
+      <c r="B16" s="175" t="inlineStr">
+        <is>
+          <t>Mise en place de l'architecture API REST</t>
+        </is>
+      </c>
+      <c r="C16" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="175" t="n"/>
+      <c r="B17" s="175" t="inlineStr">
+        <is>
+          <t>Authentification et gestion des rôles RH / admin</t>
+        </is>
+      </c>
+      <c r="C17" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="179" t="n"/>
+      <c r="B18" s="179" t="inlineStr">
+        <is>
+          <t>FRONT-OFFICE / INTERFACE</t>
+        </is>
+      </c>
+      <c r="C18" s="179" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="175" t="n"/>
+      <c r="B19" s="175" t="inlineStr">
+        <is>
+          <t>Installation de React avec Vite et structure de navigation</t>
+        </is>
+      </c>
+      <c r="C19" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="175" t="n"/>
+      <c r="B20" s="175" t="inlineStr">
+        <is>
+          <t>Intégration de la mise en page générale du back-office</t>
+        </is>
+      </c>
+      <c r="C20" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="175" t="n"/>
+      <c r="B21" s="175" t="inlineStr">
+        <is>
+          <t>Tests et debug</t>
+        </is>
+      </c>
+      <c r="C21" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="177" t="n"/>
+      <c r="B22" s="177" t="inlineStr">
+        <is>
+          <t>Sous-total</t>
+        </is>
+      </c>
+      <c r="C22" s="178">
+        <f>SUM(C13:C21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="174" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="B23" s="174" t="inlineStr">
+        <is>
+          <t>Gestion des offres, directions et domaines</t>
+        </is>
+      </c>
+      <c r="C23" s="174" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="179" t="n"/>
+      <c r="B24" s="179" t="inlineStr">
+        <is>
+          <t>BACK-OFFICE</t>
+        </is>
+      </c>
+      <c r="C24" s="179" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="175" t="n"/>
+      <c r="B25" s="175" t="inlineStr">
+        <is>
+          <t>CRUD des directions</t>
+        </is>
+      </c>
+      <c r="C25" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="175" t="n"/>
+      <c r="B26" s="175" t="inlineStr">
+        <is>
+          <t>CRUD des domaines et validation des domaines en attente</t>
+        </is>
+      </c>
+      <c r="C26" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="175" t="n"/>
+      <c r="B27" s="175" t="inlineStr">
+        <is>
+          <t>CRUD des offres d'emploi</t>
+        </is>
+      </c>
+      <c r="C27" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="175" t="n"/>
+      <c r="B28" s="175" t="inlineStr">
+        <is>
+          <t>Gestion du statut des offres : brouillon, publiée, clôturée</t>
+        </is>
+      </c>
+      <c r="C28" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="175" t="n"/>
+      <c r="B29" s="175" t="inlineStr">
+        <is>
+          <t>Gestion du profil, des missions et des formations requises</t>
+        </is>
+      </c>
+      <c r="C29" s="176" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1" s="77">
-      <c r="A11" s="156" t="n"/>
-      <c r="B11" s="156" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="175" t="n"/>
+      <c r="B30" s="175" t="inlineStr">
+        <is>
+          <t>Gestion des compétences requises par offre</t>
+        </is>
+      </c>
+      <c r="C30" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="179" t="n"/>
+      <c r="B31" s="179" t="inlineStr">
+        <is>
+          <t>FRONT-OFFICE / API</t>
+        </is>
+      </c>
+      <c r="C31" s="179" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="175" t="n"/>
+      <c r="B32" s="175" t="inlineStr">
+        <is>
+          <t>Affichage des offres publiées et génération du lien de candidature</t>
+        </is>
+      </c>
+      <c r="C32" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="175" t="n"/>
+      <c r="B33" s="175" t="inlineStr">
+        <is>
+          <t>Tests et debug</t>
+        </is>
+      </c>
+      <c r="C33" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="177" t="n"/>
+      <c r="B34" s="177" t="inlineStr">
         <is>
           <t>Sous-total</t>
         </is>
       </c>
-      <c r="C11" s="157">
-        <f>SUM(C5:C10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1" s="77">
-      <c r="A12" s="153" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="B12" s="154" t="inlineStr">
-        <is>
-          <t>Socle technique, sécurité et référentiels de base</t>
-        </is>
-      </c>
-      <c r="C12" s="153" t="n"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" s="77">
-      <c r="A13" s="158" t="n"/>
-      <c r="B13" s="158" t="inlineStr">
-        <is>
-          <t>BACK-OFFICE / API</t>
-        </is>
-      </c>
-      <c r="C13" s="159" t="n"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" s="77">
-      <c r="A14" s="151" t="n"/>
-      <c r="B14" s="151" t="inlineStr">
-        <is>
-          <t>Configuration du projet Laravel et de l'environnement PostgreSQL</t>
-        </is>
-      </c>
-      <c r="C14" s="155" t="n">
+      <c r="C34" s="178">
+        <f>SUM(C24:C33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="174" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B35" s="174" t="inlineStr">
+        <is>
+          <t>Dépôt et réception des candidatures</t>
+        </is>
+      </c>
+      <c r="C35" s="174" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="179" t="n"/>
+      <c r="B36" s="179" t="inlineStr">
+        <is>
+          <t>FRONT-OFFICE</t>
+        </is>
+      </c>
+      <c r="C36" s="179" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="175" t="n"/>
+      <c r="B37" s="175" t="inlineStr">
+        <is>
+          <t>Formulaire de candidature sur offre (temporaire)</t>
+        </is>
+      </c>
+      <c r="C37" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="175" t="n"/>
+      <c r="B38" s="175" t="inlineStr">
+        <is>
+          <t>Formulaire de candidature spontanée avec domaine (temporaire)</t>
+        </is>
+      </c>
+      <c r="C38" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="175" t="n"/>
+      <c r="B39" s="175" t="inlineStr">
+        <is>
+          <t>Upload des CV, photos et documents</t>
+        </is>
+      </c>
+      <c r="C39" s="176" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1" s="77">
-      <c r="A15" s="151" t="n"/>
-      <c r="B15" s="151" t="inlineStr">
-        <is>
-          <t>Mise en place des migrations principales et des seeders</t>
-        </is>
-      </c>
-      <c r="C15" s="155" t="n">
+    <row r="40">
+      <c r="A40" s="179" t="n"/>
+      <c r="B40" s="179" t="inlineStr">
+        <is>
+          <t>BACK-OFFICE</t>
+        </is>
+      </c>
+      <c r="C40" s="179" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="175" t="n"/>
+      <c r="B41" s="175" t="inlineStr">
+        <is>
+          <t>Saisie manuelle d'une candidature par un RH</t>
+        </is>
+      </c>
+      <c r="C41" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="179" t="n"/>
+      <c r="B42" s="179" t="inlineStr">
+        <is>
+          <t>API / SERVICES</t>
+        </is>
+      </c>
+      <c r="C42" s="179" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="175" t="n"/>
+      <c r="B43" s="175" t="inlineStr">
+        <is>
+          <t>Détection d'un candidat existant et dédoublonnage par email</t>
+        </is>
+      </c>
+      <c r="C43" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="175" t="n"/>
+      <c r="B44" s="175" t="inlineStr">
+        <is>
+          <t>Création transactionnelle : candidat, candidature, statut initial, historique</t>
+        </is>
+      </c>
+      <c r="C44" s="176" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="175" t="n"/>
+      <c r="B45" s="175" t="inlineStr">
+        <is>
+          <t>Préparation de la réception/import depuis le site externe</t>
+        </is>
+      </c>
+      <c r="C45" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="175" t="n"/>
+      <c r="B46" s="175" t="inlineStr">
+        <is>
+          <t>Tests et debug</t>
+        </is>
+      </c>
+      <c r="C46" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="177" t="n"/>
+      <c r="B47" s="177" t="inlineStr">
+        <is>
+          <t>Sous-total</t>
+        </is>
+      </c>
+      <c r="C47" s="178">
+        <f>SUM(C36:C46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="174" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B48" s="174" t="inlineStr">
+        <is>
+          <t>Gestion RH des candidatures et fiche candidat</t>
+        </is>
+      </c>
+      <c r="C48" s="174" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="179" t="n"/>
+      <c r="B49" s="179" t="inlineStr">
+        <is>
+          <t>BACK-OFFICE</t>
+        </is>
+      </c>
+      <c r="C49" s="179" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="175" t="n"/>
+      <c r="B50" s="175" t="inlineStr">
+        <is>
+          <t>Liste générale des candidatures avec pagination</t>
+        </is>
+      </c>
+      <c r="C50" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="175" t="n"/>
+      <c r="B51" s="175" t="inlineStr">
+        <is>
+          <t>Recherche et filtres : statut, direction, période, canal, type</t>
+        </is>
+      </c>
+      <c r="C51" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="175" t="n"/>
+      <c r="B52" s="175" t="inlineStr">
+        <is>
+          <t>Gestion des candidatures sur offre : Direction -&gt; Offre -&gt; Candidats</t>
+        </is>
+      </c>
+      <c r="C52" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="175" t="n"/>
+      <c r="B53" s="175" t="inlineStr">
+        <is>
+          <t>Gestion des candidatures spontanées : Direction -&gt; Domaine -&gt; Candidatures</t>
+        </is>
+      </c>
+      <c r="C53" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="175" t="n"/>
+      <c r="B54" s="175" t="inlineStr">
+        <is>
+          <t>Fiche candidat : informations, documents, historique statuts et communications</t>
+        </is>
+      </c>
+      <c r="C54" s="176" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="175" t="n"/>
+      <c r="B55" s="175" t="inlineStr">
+        <is>
+          <t>Changement de statut avec commentaire et historique</t>
+        </is>
+      </c>
+      <c r="C55" s="176" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1" s="77">
-      <c r="A16" s="151" t="n"/>
-      <c r="B16" s="151" t="inlineStr">
-        <is>
-          <t>Mise en place de l'architecture API REST</t>
-        </is>
-      </c>
-      <c r="C16" s="155" t="n">
+    <row r="56">
+      <c r="A56" s="175" t="n"/>
+      <c r="B56" s="175" t="inlineStr">
+        <is>
+          <t>Export PDF de la fiche candidat</t>
+        </is>
+      </c>
+      <c r="C56" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="175" t="n"/>
+      <c r="B57" s="175" t="inlineStr">
+        <is>
+          <t>Tests et debug</t>
+        </is>
+      </c>
+      <c r="C57" s="176" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1" s="77">
-      <c r="A17" s="151" t="n"/>
-      <c r="B17" s="151" t="inlineStr">
-        <is>
-          <t>Authentification et gestion des rôles RH / admin / manager</t>
-        </is>
-      </c>
-      <c r="C17" s="155" t="n">
+    <row r="58">
+      <c r="A58" s="177" t="n"/>
+      <c r="B58" s="177" t="inlineStr">
+        <is>
+          <t>Sous-total</t>
+        </is>
+      </c>
+      <c r="C58" s="178">
+        <f>SUM(C49:C57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="174" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="B59" s="174" t="inlineStr">
+        <is>
+          <t>Vivier, compétences et validation CV</t>
+        </is>
+      </c>
+      <c r="C59" s="174" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="179" t="n"/>
+      <c r="B60" s="179" t="inlineStr">
+        <is>
+          <t>BACK-OFFICE</t>
+        </is>
+      </c>
+      <c r="C60" s="179" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="175" t="n"/>
+      <c r="B61" s="175" t="inlineStr">
+        <is>
+          <t>Gestion du vivier : ajout, retrait, consultation</t>
+        </is>
+      </c>
+      <c r="C61" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="175" t="n"/>
+      <c r="B62" s="175" t="inlineStr">
+        <is>
+          <t>Recherche dans le vivier par compétence, domaine et direction</t>
+        </is>
+      </c>
+      <c r="C62" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="175" t="n"/>
+      <c r="B63" s="175" t="inlineStr">
+        <is>
+          <t>CRUD du référentiel des compétences</t>
+        </is>
+      </c>
+      <c r="C63" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="175" t="n"/>
+      <c r="B64" s="175" t="inlineStr">
+        <is>
+          <t>Gestion manuelle des compétences, expériences et formations candidat</t>
+        </is>
+      </c>
+      <c r="C64" s="176" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="179" t="n"/>
+      <c r="B65" s="179" t="inlineStr">
+        <is>
+          <t>OCR / IA</t>
+        </is>
+      </c>
+      <c r="C65" s="179" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="175" t="n"/>
+      <c r="B66" s="175" t="inlineStr">
+        <is>
+          <t>Intégration FastAPI et extraction OCR avec PaddleOCR</t>
+        </is>
+      </c>
+      <c r="C66" s="176" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1" s="77">
-      <c r="A18" s="158" t="n"/>
-      <c r="B18" s="158" t="inlineStr">
-        <is>
-          <t>FRONT-OFFICE / INTERFACE</t>
-        </is>
-      </c>
-      <c r="C18" s="159" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" s="77">
-      <c r="A19" s="151" t="n"/>
-      <c r="B19" s="151" t="inlineStr">
-        <is>
-          <t>Installation de React avec Vite et structure de navigation</t>
-        </is>
-      </c>
-      <c r="C19" s="155" t="n">
+    <row r="67">
+      <c r="A67" s="175" t="n"/>
+      <c r="B67" s="175" t="inlineStr">
+        <is>
+          <t>Extraction des compétences, expériences et formations depuis le CV</t>
+        </is>
+      </c>
+      <c r="C67" s="176" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="175" t="n"/>
+      <c r="B68" s="175" t="inlineStr">
+        <is>
+          <t>Validation, correction et rejet des données extraites</t>
+        </is>
+      </c>
+      <c r="C68" s="176" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="175" t="n"/>
+      <c r="B69" s="175" t="inlineStr">
+        <is>
+          <t>Tests et debug</t>
+        </is>
+      </c>
+      <c r="C69" s="176" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1" s="77">
-      <c r="A20" s="151" t="n"/>
-      <c r="B20" s="151" t="inlineStr">
-        <is>
-          <t>Intégration de la mise en page générale du back-office</t>
-        </is>
-      </c>
-      <c r="C20" s="155" t="n">
+    <row r="70">
+      <c r="A70" s="177" t="n"/>
+      <c r="B70" s="177" t="inlineStr">
+        <is>
+          <t>Sous-total</t>
+        </is>
+      </c>
+      <c r="C70" s="178">
+        <f>SUM(C60:C69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="174" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="B71" s="174" t="inlineStr">
+        <is>
+          <t>Rendez-vous, communications, automatisation et modèles</t>
+        </is>
+      </c>
+      <c r="C71" s="174" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="179" t="n"/>
+      <c r="B72" s="179" t="inlineStr">
+        <is>
+          <t>BACK-OFFICE</t>
+        </is>
+      </c>
+      <c r="C72" s="179" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="175" t="n"/>
+      <c r="B73" s="175" t="inlineStr">
+        <is>
+          <t>CRUD des rendez-vous : test, entretien, statut, mode, responsable</t>
+        </is>
+      </c>
+      <c r="C73" s="176" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="175" t="n"/>
+      <c r="B74" s="175" t="inlineStr">
+        <is>
+          <t>Vue agenda par utilisateur, candidature et période</t>
+        </is>
+      </c>
+      <c r="C74" s="176" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1" s="77">
-      <c r="A21" s="151" t="n"/>
-      <c r="B21" s="151" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="175" t="n"/>
+      <c r="B75" s="175" t="inlineStr">
+        <is>
+          <t>Communication liée aux rendez-vous</t>
+        </is>
+      </c>
+      <c r="C75" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="175" t="n"/>
+      <c r="B76" s="175" t="inlineStr">
+        <is>
+          <t>CRUD des modèles de communication</t>
+        </is>
+      </c>
+      <c r="C76" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="175" t="n"/>
+      <c r="B77" s="175" t="inlineStr">
+        <is>
+          <t>Accusé de réception et première communication automatique</t>
+        </is>
+      </c>
+      <c r="C77" s="176" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="175" t="n"/>
+      <c r="B78" s="175" t="inlineStr">
+        <is>
+          <t>Activation, désactivation et configuration de l'envoi automatique</t>
+        </is>
+      </c>
+      <c r="C78" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="179" t="n"/>
+      <c r="B79" s="179" t="inlineStr">
+        <is>
+          <t>API / SERVICES &amp; AUTOMATISATION</t>
+        </is>
+      </c>
+      <c r="C79" s="179" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="175" t="n"/>
+      <c r="B80" s="175" t="inlineStr">
+        <is>
+          <t>Récupération et ingestion des candidatures par E-mail via n8n &amp; FastAPI</t>
+        </is>
+      </c>
+      <c r="C80" s="176" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="175" t="n"/>
+      <c r="B81" s="175" t="inlineStr">
+        <is>
+          <t>Automatisation n8n : classification, routage, switch offre/spontanée et import</t>
+        </is>
+      </c>
+      <c r="C81" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="175" t="n"/>
+      <c r="B82" s="175" t="inlineStr">
+        <is>
+          <t>Envoi manuel, historique des communications et préparation des rappels</t>
+        </is>
+      </c>
+      <c r="C82" s="176" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="175" t="n"/>
+      <c r="B83" s="175" t="inlineStr">
+        <is>
+          <t>Log et Journalisation des actions RH (Audit Log)</t>
+        </is>
+      </c>
+      <c r="C83" s="176" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="175" t="n"/>
+      <c r="B84" s="175" t="inlineStr">
         <is>
           <t>Tests et debug</t>
         </is>
       </c>
-      <c r="C21" s="155" t="n">
+      <c r="C84" s="176" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1" s="77">
-      <c r="A22" s="156" t="n"/>
-      <c r="B22" s="156" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="177" t="n"/>
+      <c r="B85" s="177" t="inlineStr">
         <is>
           <t>Sous-total</t>
         </is>
       </c>
-      <c r="C22" s="157">
-        <f>SUM(C14:C21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1" s="77">
-      <c r="A23" s="153" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="B23" s="154" t="inlineStr">
-        <is>
-          <t>Gestion des offres, directions et domaines</t>
-        </is>
-      </c>
-      <c r="C23" s="153" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" s="77">
-      <c r="A24" s="158" t="n"/>
-      <c r="B24" s="158" t="inlineStr">
+      <c r="C85" s="178">
+        <f>SUM(C72:C84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="174" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
+      </c>
+      <c r="B86" s="174" t="inlineStr">
+        <is>
+          <t>Dashboard, recherche avancée, matching, audit logs et finalisation</t>
+        </is>
+      </c>
+      <c r="C86" s="174" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="179" t="n"/>
+      <c r="B87" s="179" t="inlineStr">
         <is>
           <t>BACK-OFFICE</t>
         </is>
       </c>
-      <c r="C24" s="159" t="n"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" s="77">
-      <c r="A25" s="151" t="n"/>
-      <c r="B25" s="151" t="inlineStr">
-        <is>
-          <t>CRUD des directions</t>
-        </is>
-      </c>
-      <c r="C25" s="155" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1" s="77">
-      <c r="A26" s="151" t="n"/>
-      <c r="B26" s="151" t="inlineStr">
-        <is>
-          <t>CRUD des domaines et validation des domaines en attente</t>
-        </is>
-      </c>
-      <c r="C26" s="155" t="n">
+      <c r="C87" s="179" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="175" t="n"/>
+      <c r="B88" s="175" t="inlineStr">
+        <is>
+          <t>Tableau de bord et indicateurs principaux</t>
+        </is>
+      </c>
+      <c r="C88" s="176" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1" s="77">
-      <c r="A27" s="151" t="n"/>
-      <c r="B27" s="151" t="inlineStr">
-        <is>
-          <t>CRUD des offres d'emploi</t>
-        </is>
-      </c>
-      <c r="C27" s="155" t="n">
+    <row r="89">
+      <c r="A89" s="175" t="n"/>
+      <c r="B89" s="175" t="inlineStr">
+        <is>
+          <t>Statistiques mensuelles, répartition par statut et taux de transformation</t>
+        </is>
+      </c>
+      <c r="C89" s="176" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="175" t="n"/>
+      <c r="B90" s="175" t="inlineStr">
+        <is>
+          <t>Délai moyen de traitement et filtres du dashboard</t>
+        </is>
+      </c>
+      <c r="C90" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="175" t="n"/>
+      <c r="B91" s="175" t="inlineStr">
+        <is>
+          <t>Consultation et filtrage du Journal d'Audit des actions RH</t>
+        </is>
+      </c>
+      <c r="C91" s="176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="175" t="n"/>
+      <c r="B92" s="175" t="inlineStr">
+        <is>
+          <t>Recherche avancée par mots-clés CV et compétences</t>
+        </is>
+      </c>
+      <c r="C92" s="176" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="175" t="n"/>
+      <c r="B93" s="175" t="inlineStr">
+        <is>
+          <t>Matching candidat -&gt; offre avec score simple</t>
+        </is>
+      </c>
+      <c r="C93" s="176" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1" s="77">
-      <c r="A28" s="151" t="n"/>
-      <c r="B28" s="151" t="inlineStr">
-        <is>
-          <t>Gestion du statut des offres : brouillon, publiée, clôturée</t>
-        </is>
-      </c>
-      <c r="C28" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1" s="77">
-      <c r="A29" s="151" t="n"/>
-      <c r="B29" s="151" t="inlineStr">
-        <is>
-          <t>Gestion du profil, des missions et des formations requises</t>
-        </is>
-      </c>
-      <c r="C29" s="155" t="n">
+    <row r="94">
+      <c r="A94" s="175" t="n"/>
+      <c r="B94" s="175" t="inlineStr">
+        <is>
+          <t>Tests fonctionnels globaux, corrections et optimisation</t>
+        </is>
+      </c>
+      <c r="C94" s="176" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1" s="77">
-      <c r="A30" s="151" t="n"/>
-      <c r="B30" s="151" t="inlineStr">
-        <is>
-          <t>Gestion des compétences requises par offre</t>
-        </is>
-      </c>
-      <c r="C30" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1" s="77">
-      <c r="A31" s="158" t="n"/>
-      <c r="B31" s="158" t="inlineStr">
-        <is>
-          <t>FRONT-OFFICE / API</t>
-        </is>
-      </c>
-      <c r="C31" s="159" t="n"/>
-    </row>
-    <row r="32" ht="20" customHeight="1" s="77">
-      <c r="A32" s="151" t="n"/>
-      <c r="B32" s="151" t="inlineStr">
-        <is>
-          <t>Affichage des offres publiées et génération du lien de candidature</t>
-        </is>
-      </c>
-      <c r="C32" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1" s="77">
-      <c r="A33" s="151" t="n"/>
-      <c r="B33" s="151" t="inlineStr">
-        <is>
-          <t>Tests et debug</t>
-        </is>
-      </c>
-      <c r="C33" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1" s="77">
-      <c r="A34" s="156" t="n"/>
-      <c r="B34" s="156" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="175" t="n"/>
+      <c r="B95" s="175" t="inlineStr">
+        <is>
+          <t>Documentation et préparation du déploiement</t>
+        </is>
+      </c>
+      <c r="C95" s="176" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="177" t="n"/>
+      <c r="B96" s="177" t="inlineStr">
         <is>
           <t>Sous-total</t>
         </is>
       </c>
-      <c r="C34" s="157">
-        <f>SUM(C25:C33)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="24" customHeight="1" s="77">
-      <c r="A35" s="153" t="inlineStr">
-        <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="B35" s="154" t="inlineStr">
-        <is>
-          <t>Dépôt et réception des candidatures</t>
-        </is>
-      </c>
-      <c r="C35" s="153" t="n"/>
-    </row>
-    <row r="36" ht="20" customHeight="1" s="77">
-      <c r="A36" s="158" t="n"/>
-      <c r="B36" s="158" t="inlineStr">
-        <is>
-          <t>FRONT-OFFICE</t>
-        </is>
-      </c>
-      <c r="C36" s="159" t="n"/>
-    </row>
-    <row r="37" ht="20" customHeight="1" s="77">
-      <c r="A37" s="151" t="n"/>
-      <c r="B37" s="151" t="inlineStr">
-        <is>
-          <t>Formulaire de candidature sur offre</t>
-        </is>
-      </c>
-      <c r="C37" s="155" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1" s="77">
-      <c r="A38" s="151" t="n"/>
-      <c r="B38" s="151" t="inlineStr">
-        <is>
-          <t>Formulaire de candidature spontanée avec domaine ou autre domaine</t>
-        </is>
-      </c>
-      <c r="C38" s="155" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1" s="77">
-      <c r="A39" s="151" t="n"/>
-      <c r="B39" s="151" t="inlineStr">
-        <is>
-          <t>Upload des CV, photos et documents</t>
-        </is>
-      </c>
-      <c r="C39" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1" s="77">
-      <c r="A40" s="158" t="n"/>
-      <c r="B40" s="158" t="inlineStr">
-        <is>
-          <t>BACK-OFFICE</t>
-        </is>
-      </c>
-      <c r="C40" s="159" t="n"/>
-    </row>
-    <row r="41" ht="20" customHeight="1" s="77">
-      <c r="A41" s="151" t="n"/>
-      <c r="B41" s="151" t="inlineStr">
-        <is>
-          <t>Saisie manuelle d'une candidature par un RH</t>
-        </is>
-      </c>
-      <c r="C41" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1" s="77">
-      <c r="A42" s="158" t="n"/>
-      <c r="B42" s="158" t="inlineStr">
-        <is>
-          <t>API / SERVICES</t>
-        </is>
-      </c>
-      <c r="C42" s="159" t="n"/>
-    </row>
-    <row r="43" ht="20" customHeight="1" s="77">
-      <c r="A43" s="151" t="n"/>
-      <c r="B43" s="151" t="inlineStr">
-        <is>
-          <t>Détection d'un candidat existant et dédoublonnage par email</t>
-        </is>
-      </c>
-      <c r="C43" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" ht="20" customHeight="1" s="77">
-      <c r="A44" s="151" t="n"/>
-      <c r="B44" s="151" t="inlineStr">
-        <is>
-          <t>Création transactionnelle : candidat, candidature, statut initial, historique</t>
-        </is>
-      </c>
-      <c r="C44" s="155" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1" s="77">
-      <c r="A45" s="151" t="n"/>
-      <c r="B45" s="151" t="inlineStr">
-        <is>
-          <t>Préparation de la réception/import depuis le site externe</t>
-        </is>
-      </c>
-      <c r="C45" s="155" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1" s="77">
-      <c r="A46" s="151" t="n"/>
-      <c r="B46" s="151" t="inlineStr">
-        <is>
-          <t>Accusé de réception et première communication automatique</t>
-        </is>
-      </c>
-      <c r="C46" s="155" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1" s="77">
-      <c r="A47" s="151" t="n"/>
-      <c r="B47" s="151" t="inlineStr">
-        <is>
-          <t>Tests et debug</t>
-        </is>
-      </c>
-      <c r="C47" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1" s="77">
-      <c r="A48" s="156" t="n"/>
-      <c r="B48" s="156" t="inlineStr">
-        <is>
-          <t>Sous-total</t>
-        </is>
-      </c>
-      <c r="C48" s="157">
-        <f>SUM(C37:C47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="24" customHeight="1" s="77">
-      <c r="A49" s="153" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
-      </c>
-      <c r="B49" s="154" t="inlineStr">
-        <is>
-          <t>Gestion RH des candidatures et fiche candidat</t>
-        </is>
-      </c>
-      <c r="C49" s="153" t="n"/>
-    </row>
-    <row r="50" ht="20" customHeight="1" s="77">
-      <c r="A50" s="158" t="n"/>
-      <c r="B50" s="158" t="inlineStr">
-        <is>
-          <t>BACK-OFFICE</t>
-        </is>
-      </c>
-      <c r="C50" s="159" t="n"/>
-    </row>
-    <row r="51" ht="20" customHeight="1" s="77">
-      <c r="A51" s="151" t="n"/>
-      <c r="B51" s="151" t="inlineStr">
-        <is>
-          <t>Liste générale des candidatures avec pagination</t>
-        </is>
-      </c>
-      <c r="C51" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" ht="20" customHeight="1" s="77">
-      <c r="A52" s="151" t="n"/>
-      <c r="B52" s="151" t="inlineStr">
-        <is>
-          <t>Recherche et filtres : statut, direction, période, canal, type</t>
-        </is>
-      </c>
-      <c r="C52" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1" s="77">
-      <c r="A53" s="151" t="n"/>
-      <c r="B53" s="151" t="inlineStr">
-        <is>
-          <t>Gestion des candidatures sur offre : Direction -&gt; Offre -&gt; Candidats</t>
-        </is>
-      </c>
-      <c r="C53" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" ht="20" customHeight="1" s="77">
-      <c r="A54" s="151" t="n"/>
-      <c r="B54" s="151" t="inlineStr">
-        <is>
-          <t>Gestion des candidatures spontanées : Direction -&gt; Domaine -&gt; Candidatures</t>
-        </is>
-      </c>
-      <c r="C54" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" ht="20" customHeight="1" s="77">
-      <c r="A55" s="151" t="n"/>
-      <c r="B55" s="151" t="inlineStr">
-        <is>
-          <t>Fiche candidat : informations, documents, statut, historique statuts et communications</t>
-        </is>
-      </c>
-      <c r="C55" s="155" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" ht="20" customHeight="1" s="77">
-      <c r="A56" s="151" t="n"/>
-      <c r="B56" s="151" t="inlineStr">
-        <is>
-          <t>Changement de statut avec commentaire et historique</t>
-        </is>
-      </c>
-      <c r="C56" s="155" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1" s="77">
-      <c r="A57" s="151" t="n"/>
-      <c r="B57" s="151" t="inlineStr">
-        <is>
-          <t>Export PDF de la fiche candidat</t>
-        </is>
-      </c>
-      <c r="C57" s="155" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="58" ht="20" customHeight="1" s="77">
-      <c r="A58" s="151" t="n"/>
-      <c r="B58" s="151" t="inlineStr">
-        <is>
-          <t>Tests et debug</t>
-        </is>
-      </c>
-      <c r="C58" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" ht="20" customHeight="1" s="77">
-      <c r="A59" s="156" t="n"/>
-      <c r="B59" s="156" t="inlineStr">
-        <is>
-          <t>Sous-total</t>
-        </is>
-      </c>
-      <c r="C59" s="157">
-        <f>SUM(C51:C58)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="24" customHeight="1" s="77">
-      <c r="A60" s="153" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
-      </c>
-      <c r="B60" s="154" t="inlineStr">
-        <is>
-          <t>Vivier, compétences et validation CV</t>
-        </is>
-      </c>
-      <c r="C60" s="153" t="n"/>
-    </row>
-    <row r="61" ht="20" customHeight="1" s="77">
-      <c r="A61" s="158" t="n"/>
-      <c r="B61" s="158" t="inlineStr">
-        <is>
-          <t>BACK-OFFICE</t>
-        </is>
-      </c>
-      <c r="C61" s="159" t="n"/>
-    </row>
-    <row r="62" ht="20" customHeight="1" s="77">
-      <c r="A62" s="151" t="n"/>
-      <c r="B62" s="151" t="inlineStr">
-        <is>
-          <t>Gestion du vivier : ajout, retrait, consultation</t>
-        </is>
-      </c>
-      <c r="C62" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" ht="20" customHeight="1" s="77">
-      <c r="A63" s="151" t="n"/>
-      <c r="B63" s="151" t="inlineStr">
-        <is>
-          <t>Recherche dans le vivier par compétence, domaine et direction</t>
-        </is>
-      </c>
-      <c r="C63" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" ht="20" customHeight="1" s="77">
-      <c r="A64" s="151" t="n"/>
-      <c r="B64" s="151" t="inlineStr">
-        <is>
-          <t>CRUD du référentiel des compétences</t>
-        </is>
-      </c>
-      <c r="C64" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1" s="77">
-      <c r="A65" s="151" t="n"/>
-      <c r="B65" s="151" t="inlineStr">
-        <is>
-          <t>Gestion manuelle des compétences, expériences et formations candidat</t>
-        </is>
-      </c>
-      <c r="C65" s="155" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="66" ht="20" customHeight="1" s="77">
-      <c r="A66" s="158" t="n"/>
-      <c r="B66" s="158" t="inlineStr">
-        <is>
-          <t>OCR / IA</t>
-        </is>
-      </c>
-      <c r="C66" s="159" t="n"/>
-    </row>
-    <row r="67" ht="20" customHeight="1" s="77">
-      <c r="A67" s="151" t="n"/>
-      <c r="B67" s="151" t="inlineStr">
-        <is>
-          <t>Intégration FastAPI et extraction OCR avec PaddleOCR</t>
-        </is>
-      </c>
-      <c r="C67" s="155" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="68" ht="20" customHeight="1" s="77">
-      <c r="A68" s="151" t="n"/>
-      <c r="B68" s="151" t="inlineStr">
-        <is>
-          <t>Extraction des compétences, expériences et formations depuis le CV</t>
-        </is>
-      </c>
-      <c r="C68" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" ht="20" customHeight="1" s="77">
-      <c r="A69" s="151" t="n"/>
-      <c r="B69" s="151" t="inlineStr">
-        <is>
-          <t>Validation, correction et rejet des données extraites</t>
-        </is>
-      </c>
-      <c r="C69" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" ht="20" customHeight="1" s="77">
-      <c r="A70" s="151" t="n"/>
-      <c r="B70" s="151" t="inlineStr">
-        <is>
-          <t>Tests et debug</t>
-        </is>
-      </c>
-      <c r="C70" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" ht="20" customHeight="1" s="77">
-      <c r="A71" s="156" t="n"/>
-      <c r="B71" s="156" t="inlineStr">
-        <is>
-          <t>Sous-total</t>
-        </is>
-      </c>
-      <c r="C71" s="157">
-        <f>SUM(C62:C70)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" ht="24" customHeight="1" s="77">
-      <c r="A72" s="153" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
-      </c>
-      <c r="B72" s="154" t="inlineStr">
-        <is>
-          <t>Rendez-vous, communications et modèles</t>
-        </is>
-      </c>
-      <c r="C72" s="153" t="n"/>
-    </row>
-    <row r="73" ht="20" customHeight="1" s="77">
-      <c r="A73" s="158" t="n"/>
-      <c r="B73" s="158" t="inlineStr">
-        <is>
-          <t>BACK-OFFICE</t>
-        </is>
-      </c>
-      <c r="C73" s="159" t="n"/>
-    </row>
-    <row r="74" ht="20" customHeight="1" s="77">
-      <c r="A74" s="151" t="n"/>
-      <c r="B74" s="151" t="inlineStr">
-        <is>
-          <t>CRUD des rendez-vous : test, entretien, statut, mode, responsable</t>
-        </is>
-      </c>
-      <c r="C74" s="155" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1" s="77">
-      <c r="A75" s="151" t="n"/>
-      <c r="B75" s="151" t="inlineStr">
-        <is>
-          <t>Vue agenda par utilisateur, candidature et période</t>
-        </is>
-      </c>
-      <c r="C75" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76" ht="20" customHeight="1" s="77">
-      <c r="A76" s="151" t="n"/>
-      <c r="B76" s="151" t="inlineStr">
-        <is>
-          <t>Communication liée aux rendez-vous</t>
-        </is>
-      </c>
-      <c r="C76" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" ht="20" customHeight="1" s="77">
-      <c r="A77" s="151" t="n"/>
-      <c r="B77" s="151" t="inlineStr">
-        <is>
-          <t>CRUD des modèles de communication</t>
-        </is>
-      </c>
-      <c r="C77" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78" ht="20" customHeight="1" s="77">
-      <c r="A78" s="151" t="n"/>
-      <c r="B78" s="151" t="inlineStr">
-        <is>
-          <t>Activation, désactivation et configuration de l'envoi automatique</t>
-        </is>
-      </c>
-      <c r="C78" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79" ht="20" customHeight="1" s="77">
-      <c r="A79" s="158" t="n"/>
-      <c r="B79" s="158" t="inlineStr">
-        <is>
-          <t>API / SERVICES</t>
-        </is>
-      </c>
-      <c r="C79" s="159" t="n"/>
-    </row>
-    <row r="80" ht="20" customHeight="1" s="77">
-      <c r="A80" s="151" t="n"/>
-      <c r="B80" s="151" t="inlineStr">
-        <is>
-          <t>Envoi manuel, historique des communications et préparation des rappels</t>
-        </is>
-      </c>
-      <c r="C80" s="155" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="81" ht="20" customHeight="1" s="77">
-      <c r="A81" s="151" t="n"/>
-      <c r="B81" s="151" t="inlineStr">
-        <is>
-          <t>Tests et debug</t>
-        </is>
-      </c>
-      <c r="C81" s="155" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="82" ht="20" customHeight="1" s="77">
-      <c r="A82" s="156" t="n"/>
-      <c r="B82" s="156" t="inlineStr">
-        <is>
-          <t>Sous-total</t>
-        </is>
-      </c>
-      <c r="C82" s="157">
-        <f>SUM(C74:C81)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83" ht="24" customHeight="1" s="77">
-      <c r="A83" s="153" t="inlineStr">
-        <is>
-          <t>Sprint 7</t>
-        </is>
-      </c>
-      <c r="B83" s="154" t="inlineStr">
-        <is>
-          <t>Dashboard, recherche avancée, matching et finalisation</t>
-        </is>
-      </c>
-      <c r="C83" s="153" t="n"/>
-    </row>
-    <row r="84" ht="20" customHeight="1" s="77">
-      <c r="A84" s="158" t="n"/>
-      <c r="B84" s="158" t="inlineStr">
-        <is>
-          <t>BACK-OFFICE</t>
-        </is>
-      </c>
-      <c r="C84" s="159" t="n"/>
-    </row>
-    <row r="85" ht="20" customHeight="1" s="77">
-      <c r="A85" s="151" t="n"/>
-      <c r="B85" s="151" t="inlineStr">
-        <is>
-          <t>Tableau de bord et indicateurs principaux</t>
-        </is>
-      </c>
-      <c r="C85" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" ht="20" customHeight="1" s="77">
-      <c r="A86" s="151" t="n"/>
-      <c r="B86" s="151" t="inlineStr">
-        <is>
-          <t>Statistiques mensuelles, répartition par statut et taux de transformation</t>
-        </is>
-      </c>
-      <c r="C86" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87" ht="20" customHeight="1" s="77">
-      <c r="A87" s="151" t="n"/>
-      <c r="B87" s="151" t="inlineStr">
-        <is>
-          <t>Délai moyen de traitement et filtres du dashboard</t>
-        </is>
-      </c>
-      <c r="C87" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" ht="20" customHeight="1" s="77">
-      <c r="A88" s="151" t="n"/>
-      <c r="B88" s="151" t="inlineStr">
-        <is>
-          <t>Recherche avancée par mots-clés CV et compétences</t>
-        </is>
-      </c>
-      <c r="C88" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" ht="20" customHeight="1" s="77">
-      <c r="A89" s="151" t="n"/>
-      <c r="B89" s="151" t="inlineStr">
-        <is>
-          <t>Matching candidat -&gt; offre avec score simple</t>
-        </is>
-      </c>
-      <c r="C89" s="155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" ht="20" customHeight="1" s="77">
-      <c r="A90" s="151" t="n"/>
-      <c r="B90" s="151" t="inlineStr">
-        <is>
-          <t>Tests fonctionnels globaux, corrections et optimisation</t>
-        </is>
-      </c>
-      <c r="C90" s="155" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="91" ht="20" customHeight="1" s="77">
-      <c r="A91" s="151" t="n"/>
-      <c r="B91" s="151" t="inlineStr">
-        <is>
-          <t>Documentation et préparation du déploiement</t>
-        </is>
-      </c>
-      <c r="C91" s="155" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="92" ht="20" customHeight="1" s="77">
-      <c r="A92" s="156" t="n"/>
-      <c r="B92" s="156" t="inlineStr">
-        <is>
-          <t>Sous-total</t>
-        </is>
-      </c>
-      <c r="C92" s="157">
-        <f>SUM(C85:C91)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" ht="26" customHeight="1" s="77">
-      <c r="A93" s="160" t="n"/>
-      <c r="B93" s="160" t="inlineStr">
+      <c r="C96" s="178">
+        <f>SUM(C87:C95)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="180" t="n"/>
+      <c r="B97" s="180" t="inlineStr">
         <is>
           <t>Total Scope</t>
         </is>
       </c>
-      <c r="C93" s="161">
-        <f>SUM(C11,C22,C34,C48,C59,C71,C82,C92)</f>
+      <c r="C97" s="181">
+        <f>SUM(C11,C22,C34,C47,C58,C70,C85,C96)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:C93"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 

</xml_diff>